<commit_message>
New Version Updated Status
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\__Slim 4\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\__Slim 4\Web site\Final\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4E8D7F4-483B-4246-A4E3-F68343FBFBD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98B6621A-6F86-4912-B9B5-F7A06A37E714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="30">
   <si>
     <t>ID</t>
   </si>
@@ -89,6 +89,27 @@
   </si>
   <si>
     <t xml:space="preserve">Vacation </t>
+  </si>
+  <si>
+    <t>Dev &amp; Testing Status</t>
+  </si>
+  <si>
+    <t>Historical Data Status</t>
+  </si>
+  <si>
+    <t>In-Progress</t>
+  </si>
+  <si>
+    <t>Finished</t>
+  </si>
+  <si>
+    <t>Delayed</t>
+  </si>
+  <si>
+    <t>Not-Started</t>
+  </si>
+  <si>
+    <t>On-Hold</t>
   </si>
 </sst>
 </file>
@@ -450,7 +471,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -458,13 +479,15 @@
     <col min="3" max="3" width="18" customWidth="1"/>
     <col min="4" max="4" width="22.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="22" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="23.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="22.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20" customWidth="1"/>
+    <col min="6" max="6" width="22" customWidth="1"/>
+    <col min="7" max="7" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="22.42578125" customWidth="1"/>
+    <col min="11" max="11" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -481,19 +504,25 @@
         <v>18</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="G1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -509,12 +538,16 @@
       <c r="E2" s="3">
         <v>46159</v>
       </c>
-      <c r="F2" s="2"/>
+      <c r="F2" s="3" t="s">
+        <v>25</v>
+      </c>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -530,14 +563,18 @@
       <c r="E3" s="3">
         <v>46161</v>
       </c>
-      <c r="F3" s="2"/>
+      <c r="F3" s="3" t="s">
+        <v>25</v>
+      </c>
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
-      <c r="I3" s="2" t="s">
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+      <c r="K3" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -553,20 +590,26 @@
       <c r="E4" s="3">
         <v>46173</v>
       </c>
-      <c r="F4" s="2">
+      <c r="F4" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" s="2">
         <v>7</v>
       </c>
-      <c r="G4" s="3">
+      <c r="H4" s="3">
         <v>46174</v>
       </c>
-      <c r="H4" s="3">
+      <c r="I4" s="3">
         <v>46182</v>
       </c>
-      <c r="I4" s="2">
+      <c r="J4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="K4" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>3</v>
       </c>
@@ -582,14 +625,18 @@
       <c r="E5" s="3">
         <v>46170</v>
       </c>
-      <c r="F5" s="2"/>
-      <c r="G5" s="3"/>
+      <c r="F5" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="G5" s="2"/>
       <c r="H5" s="3"/>
-      <c r="I5" s="2">
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>4</v>
       </c>
@@ -605,14 +652,18 @@
       <c r="E6" s="3">
         <v>46187</v>
       </c>
-      <c r="F6" s="2"/>
+      <c r="F6" s="3" t="s">
+        <v>28</v>
+      </c>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
-      <c r="I6" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I6" s="2"/>
+      <c r="J6" s="2"/>
+      <c r="K6" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>5</v>
       </c>
@@ -628,14 +679,18 @@
       <c r="E7" s="3">
         <v>46190</v>
       </c>
-      <c r="F7" s="2"/>
+      <c r="F7" s="3" t="s">
+        <v>29</v>
+      </c>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
-      <c r="I7" s="2">
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2">
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>6</v>
       </c>
@@ -651,14 +706,18 @@
       <c r="E8" s="3">
         <v>46196</v>
       </c>
-      <c r="F8" s="2"/>
+      <c r="F8" s="3" t="s">
+        <v>29</v>
+      </c>
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
-      <c r="I8" s="2">
+      <c r="I8" s="2"/>
+      <c r="J8" s="2"/>
+      <c r="K8" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>7</v>
       </c>
@@ -674,14 +733,18 @@
       <c r="E9" s="3">
         <v>46201</v>
       </c>
-      <c r="F9" s="2"/>
+      <c r="F9" s="3" t="s">
+        <v>26</v>
+      </c>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
-      <c r="I9" s="2">
+      <c r="I9" s="2"/>
+      <c r="J9" s="2"/>
+      <c r="K9" s="2">
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>8</v>
       </c>
@@ -697,14 +760,18 @@
       <c r="E10" s="3">
         <v>46203</v>
       </c>
-      <c r="F10" s="2"/>
+      <c r="F10" s="3" t="s">
+        <v>27</v>
+      </c>
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
-      <c r="I10" s="2">
+      <c r="I10" s="2"/>
+      <c r="J10" s="2"/>
+      <c r="K10" s="2">
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>9</v>
       </c>
@@ -720,14 +787,18 @@
       <c r="E11" s="3">
         <v>46209</v>
       </c>
-      <c r="F11" s="2"/>
+      <c r="F11" s="3" t="s">
+        <v>28</v>
+      </c>
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
-      <c r="I11" s="2">
+      <c r="I11" s="2"/>
+      <c r="J11" s="2"/>
+      <c r="K11" s="2">
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>10</v>
       </c>
@@ -743,20 +814,26 @@
       <c r="E12" s="3">
         <v>46212</v>
       </c>
-      <c r="F12" s="2">
+      <c r="F12" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="G12" s="2">
         <v>10</v>
       </c>
-      <c r="G12" s="3">
+      <c r="H12" s="3">
         <v>46215</v>
       </c>
-      <c r="H12" s="3">
+      <c r="I12" s="3">
         <v>46226</v>
       </c>
-      <c r="I12" s="2">
+      <c r="J12" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="K12" s="2">
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>11</v>
       </c>
@@ -772,14 +849,18 @@
       <c r="E13" s="3">
         <v>46233</v>
       </c>
-      <c r="F13" s="2"/>
+      <c r="F13" s="3" t="s">
+        <v>28</v>
+      </c>
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
-      <c r="I13" s="2">
+      <c r="I13" s="2"/>
+      <c r="J13" s="2"/>
+      <c r="K13" s="2">
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>12</v>
       </c>
@@ -795,13 +876,16 @@
       <c r="E14" s="3">
         <v>46238</v>
       </c>
-      <c r="F14" s="2"/>
-      <c r="I14" s="2">
+      <c r="F14" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="G14" s="2"/>
+      <c r="K14" s="2">
         <v>11</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I14">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K14">
     <sortCondition ref="A2:A14"/>
   </sortState>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>